<commit_message>
JLCPCB: colonna "JLCPCB Part #", codici esatti, U5/U7/D1/J1-J4 a mano
Dal report del BOM Tool di JLCPCB: la colonna "LCSC Part #" veniva ignorata
e i resistori abbinati a caso. Ora ogni riga ha il codice JLCPCB o l'MPN
(resistori UNI-ROYAL 0805W8F...T5E). LP2985-3.6 e 1N4148 esauriti e header
non riconosciuti passano alla lista da saldare a mano.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017fc9yPsNewCQrMK8R1c8Ls
</commit_message>
<xml_diff>
--- a/hardware/jlcpcb/BOM_JLCPCB.xlsx
+++ b/hardware/jlcpcb/BOM_JLCPCB.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,14 +434,14 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>LCSC Part #</t>
+          <t>JLCPCB Part #</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>22pF 50V 0805</t>
+          <t>CL21C220JBANNNC</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -454,12 +454,16 @@
           <t>0805</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>C1804</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1uF 100V X7R</t>
+          <t>1210B105K101NT</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -472,12 +476,16 @@
           <t>1210</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>C24365</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>100nF 100V X7R</t>
+          <t>CC1206KKX7R0BB104</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -499,7 +507,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>100nF 50V X7R</t>
+          <t>CC0805KRX7R9BB104</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -521,7 +529,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>10nF 50V 0805</t>
+          <t>CL21B103KBANNNC</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -534,12 +542,16 @@
           <t>0805</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>C1710</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>100pF 50V 0805</t>
+          <t>CL21C101JBANNNC</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -552,12 +564,16 @@
           <t>0805</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>C1790</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1uF 50V 0805</t>
+          <t>CL21B105KBFNNNE</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -570,141 +586,149 @@
           <t>0805</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>C28323</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1N4148</t>
+          <t>NCD0805R1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>DO-35 (THT)</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>C14538</t>
+          <t>C84256</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LED rosso</t>
+          <t>SRN5040-470M</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>LED 0805</t>
+          <t>SMD 5x5mm</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>C84256</t>
+          <t>C1330294</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Header 1x2 2.54mm</t>
+          <t>BFR93AE6327HTSA1</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>J1,J2,J3,J4</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Header 2.54mm 1x2 (THT)</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
+          <t>SOT-23</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>C513260</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>47uH 0.9A</t>
+          <t>MMBTH81</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>SMD 5x5mm</t>
+          <t>SOT-23</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>C1330294</t>
+          <t>C190349</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BFR93A</t>
+          <t>0805W8F1002T5E</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>R1,R10</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>SOT-23</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr"/>
+          <t>0805</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>C17414</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MMBTH81</t>
+          <t>0805W8F6802T5E</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>SOT-23</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>C190349</t>
-        </is>
-      </c>
+          <t>0805</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>10k 1% 0805</t>
+          <t>0805W8F2703T5E</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>R1,R10</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -717,12 +741,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>68k 1% 0805</t>
+          <t>0805W8F1201T5E</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -735,12 +759,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>270k 1% 0805</t>
+          <t>0805W8F1502T5E</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -753,12 +777,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1.2k 1% 0805</t>
+          <t>0805W8F1003T5E</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R6,R20</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -771,12 +795,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>15k 1% 0805</t>
+          <t>0805W8F2702T5E</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R7</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -789,12 +813,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>100k 1% 0805</t>
+          <t>0805W8F1001T5E</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>R6,R20</t>
+          <t>R8,R12,R14,R15,R16</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -807,12 +831,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>27k 1% 0805</t>
+          <t>0805W8F1801T5E</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R9</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -825,12 +849,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1k 1% 0805</t>
+          <t>0805W8F5601T5E</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>R8,R12,R14,R15,R16</t>
+          <t>R11</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -843,12 +867,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1.8k 1% 0805</t>
+          <t>0805W8F5600T5E</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>R9</t>
+          <t>R13</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -861,12 +885,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>5.6k 1% 0805</t>
+          <t>0805W8F4700T5E</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>R11</t>
+          <t>R17</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -879,12 +903,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>560 1% 0805</t>
+          <t>0805W8F100JT5E</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>R13</t>
+          <t>R18</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -897,12 +921,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>470 1% 0805</t>
+          <t>0805W8F1802T5E</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>R17</t>
+          <t>R19</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -915,12 +939,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>10 1% 0805</t>
+          <t>0805W8F820JT5E</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>R18</t>
+          <t>R21</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -933,12 +957,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>18k 1% 0805</t>
+          <t>0805W8F2203T5E</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>R19</t>
+          <t>R22</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -951,12 +975,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>82 1% 0805</t>
+          <t>0805W8F330JT5E</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>R21</t>
+          <t>R23</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -969,66 +993,78 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>220k 1% 0805</t>
+          <t>TLC555CDR</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>R22</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>0805</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr"/>
+          <t>SOIC-8</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>C6986</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>33 1% 0805</t>
+          <t>MCP1402T-E/OT</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>R23</t>
+          <t>U4</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0805</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr"/>
+          <t>SOT-23-5</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>C128573</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>TLC555CDR</t>
+          <t>MCP1825S-3302E/DB</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>U6</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>SOIC-8</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr"/>
+          <t>SOT-223</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>C148031</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>MCP1402T-E/OT</t>
+          <t>SN74LVC1G17DBVR</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>U4</t>
+          <t>U9</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1038,89 +1074,27 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>C128573</t>
+          <t>C7836</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>LP2985AIM5-3.6/NOPB</t>
+          <t>3296W-1-103LF</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>U5,U7</t>
+          <t>V1,V2</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>SOT-23-5</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>MCP1825S-3302E/DB</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>U6</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>SOT-223</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>C148031</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>SN74LVC1G17DBVR</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>U9</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>SOT-23-5</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>C7836</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>10k trimmer 3296W</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>V1,V2</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>3296W (THT)</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
+          <t>3296W</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
         <is>
           <t>C34846</t>
         </is>

</xml_diff>